<commit_message>
Cluster analysis of factoriescap_s usage 0
</commit_message>
<xml_diff>
--- a/clustering/median of 4 clusters (factoriescap_s (usage) 0).xlsx
+++ b/clustering/median of 4 clusters (factoriescap_s (usage) 0).xlsx
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>clust</t>
   </si>
@@ -89,18 +89,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -405,13 +399,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -436,16 +430,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="2">
-        <v>319996.87399999698</v>
+        <v>337263.2171999964</v>
       </c>
       <c r="C2" s="2">
-        <v>171.9999999999992</v>
+        <v>190.99999999999821</v>
       </c>
       <c r="D2" s="2">
-        <v>6.9999999999999503</v>
+        <v>7.9999999999999636</v>
       </c>
       <c r="E2" s="2">
-        <v>29.99999999999951</v>
+        <v>33.999999999999943</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -470,16 +464,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>1376076.8447999989</v>
+        <v>2172851.712599996</v>
       </c>
       <c r="C4" s="2">
-        <v>1080</v>
+        <v>2182</v>
       </c>
       <c r="D4" s="2">
-        <v>45.999999999999993</v>
+        <v>75.999999999999957</v>
       </c>
       <c r="E4" s="2">
-        <v>203.9999999999996</v>
+        <v>383.99999999999972</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -487,165 +481,19 @@
         <v>3</v>
       </c>
       <c r="B5" s="2">
-        <v>4120311.0479999962</v>
+        <v>4317554.7359999968</v>
       </c>
       <c r="C5" s="2">
-        <v>2927.9999999999991</v>
+        <v>4499</v>
       </c>
       <c r="D5" s="2">
-        <v>141.49999999999989</v>
+        <v>233</v>
       </c>
       <c r="E5" s="2">
-        <v>635.99999999999966</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>0</v>
-      </c>
-      <c r="B8" s="4">
-        <v>0</v>
-      </c>
-      <c r="C8" s="4">
-        <v>0</v>
-      </c>
-      <c r="D8" s="4">
-        <v>0</v>
-      </c>
-      <c r="E8" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
-        <v>1</v>
-      </c>
-      <c r="B9" s="3">
-        <f>B3/B$2</f>
-        <v>134.04765566053749</v>
-      </c>
-      <c r="C9" s="3">
-        <f t="shared" ref="C9:E11" si="0">C3/C$2</f>
-        <v>99.296511627907435</v>
-      </c>
-      <c r="D9" s="3">
-        <f t="shared" si="0"/>
-        <v>102.57142857142929</v>
-      </c>
-      <c r="E9" s="3">
-        <f t="shared" si="0"/>
-        <v>113.10000000000184</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>2</v>
-      </c>
-      <c r="B10" s="3">
-        <f>B4/B$2</f>
-        <v>4.3002821483812745</v>
-      </c>
-      <c r="C10" s="3">
-        <f t="shared" si="0"/>
-        <v>6.2790697674418894</v>
-      </c>
-      <c r="D10" s="3">
-        <f t="shared" si="0"/>
-        <v>6.5714285714286174</v>
-      </c>
-      <c r="E10" s="3">
-        <f t="shared" si="0"/>
-        <v>6.8000000000000975</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <v>3</v>
-      </c>
-      <c r="B11" s="3">
-        <f>B5/B$2</f>
-        <v>12.876097808380575</v>
-      </c>
-      <c r="C11" s="3">
-        <f t="shared" si="0"/>
-        <v>17.023255813953561</v>
-      </c>
-      <c r="D11" s="3">
-        <f t="shared" si="0"/>
-        <v>20.214285714285843</v>
-      </c>
-      <c r="E11" s="3">
-        <f t="shared" si="0"/>
-        <v>21.200000000000337</v>
+        <v>796.99999999999966</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:C5">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D5">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E5">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B5">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>